<commit_message>
feat: download direto imediato no scraper (requests + fallback selenium)
- Adiciona funcao baixar_arquivo_direto() que extrai o href do link
  e faz download via requests usando cookies da sessao Selenium.
- Download e salvo DIRETAMENTE no destino final, sem passar por
  temp_dl e sem depender de nova janela/popup.
- Se o download direto falhar, cai no fluxo legado (Selenium + temp_dl).
- Evita que arquivos fiquem pendentes quando o sistema fica inativo.
- Aplica melhoria tanto no scraper.py standalone quanto no
  run_scraper.py (management command Django).
</commit_message>
<xml_diff>
--- a/empresasindicato.xlsx
+++ b/empresasindicato.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Script\mediadorcct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3289D3F1-FB3D-4BEA-A497-001C7EB26B79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A360C0E6-2C5C-41FA-8949-9E4F21346245}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3885" yWindow="225" windowWidth="21570" windowHeight="15255" xr2:uid="{61B9FAB5-9018-445C-9E70-B1758252F8D9}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{61B9FAB5-9018-445C-9E70-B1758252F8D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="252">
   <si>
     <t>COMERCIAL WELINGTON LTDA</t>
   </si>
@@ -782,9 +782,6 @@
     <t>W20 INDUSTRIA E COMERCIO LTDA</t>
   </si>
   <si>
-    <t>empresa</t>
-  </si>
-  <si>
     <t>codempresa</t>
   </si>
   <si>
@@ -792,6 +789,12 @@
   </si>
   <si>
     <t>codsindicato2</t>
+  </si>
+  <si>
+    <t>nomeempresa</t>
+  </si>
+  <si>
+    <t>codsindicato3</t>
   </si>
 </sst>
 </file>
@@ -1163,30 +1166,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82DE25B6-C407-4FA0-BE77-316BD9181906}">
-  <dimension ref="A1:D249"/>
+  <dimension ref="A1:E249"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C1" t="s">
         <v>248</v>
       </c>
-      <c r="B1" t="s">
-        <v>247</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>249</v>
       </c>
-      <c r="D1" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>472</v>
       </c>
@@ -1194,7 +1200,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>551</v>
       </c>
@@ -1205,7 +1211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>567</v>
       </c>
@@ -1216,7 +1222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>84</v>
       </c>
@@ -1227,7 +1233,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>446</v>
       </c>
@@ -1238,7 +1244,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>162</v>
       </c>
@@ -1249,7 +1255,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>132</v>
       </c>
@@ -1260,7 +1266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>394</v>
       </c>
@@ -1271,7 +1277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>339</v>
       </c>
@@ -1282,7 +1288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>295</v>
       </c>
@@ -1293,7 +1299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>196</v>
       </c>
@@ -1304,7 +1310,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>517</v>
       </c>
@@ -1315,7 +1321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>511</v>
       </c>
@@ -1326,7 +1332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>513</v>
       </c>
@@ -1337,7 +1343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>223</v>
       </c>

</xml_diff>